<commit_message>
Refresh daily regional overview
</commit_message>
<xml_diff>
--- a/pipeline/reports-daily/daily-region-overview.xlsx
+++ b/pipeline/reports-daily/daily-region-overview.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sitewide" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JobG8 categories" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LIVE" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NOT LIVE" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Sitewide" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="JobG8 categories" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="LIVE" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="NOT LIVE" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sitewide'!$A$1:$B$9</definedName>
@@ -2278,38 +2278,36 @@
       <c r="B2" s="2" t="inlineStr"/>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.2 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2 / 2.2 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>4 / 3.8 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>1 / 1.1 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>1 / 0.7 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>1 / 1.0 / 0/8</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>1 / 1.0 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -2319,32 +2317,28 @@
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr"/>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>0 / 3.5 / 3/11</t>
-        </is>
+      <c r="C3" s="5" t="n">
+        <v>2</v>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>7 / 1.7 / 1/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>2 / 0.7 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr"/>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>2 / 0.5 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr"/>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>1 / 0.2 / 0/5</t>
-        </is>
+      <c r="I3" s="5" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -2354,32 +2348,28 @@
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr"/>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>1 / 1.0 / 0/11</t>
-        </is>
+      <c r="C4" s="3" t="n">
+        <v>3</v>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>3 / 2.9 / 1/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>7 / 2.6 / 1/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>2 / 1.8 / 0/8</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>5 / 2.0 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -2389,36 +2379,32 @@
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr"/>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>0 / 0.7 / 0/11</t>
-        </is>
+      <c r="C5" s="5" t="n">
+        <v>2</v>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>1 / 0.6 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>1 / 1.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr"/>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>1 / 2.0 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>1 / 0.8 / 0/8</t>
-        </is>
-      </c>
-      <c r="I5" s="4" t="inlineStr">
-        <is>
-          <t>6 / 2.4 / 1/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -2428,40 +2414,36 @@
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr"/>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>0 / 0.1 / 0/11</t>
-        </is>
+      <c r="C6" s="3" t="n">
+        <v>2</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>3 / 2.5 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>1 / 1.2 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>6 / 2.6 / 1/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>3 / 4.5 / 2/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.1 / 0/8</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>1 / 1.0 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -2471,40 +2453,36 @@
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr"/>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>0 / 0.6 / 0/11</t>
-        </is>
+      <c r="C7" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>3 / 1.5 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.2 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>3 / 1.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/8</t>
-        </is>
-      </c>
-      <c r="I7" s="4" t="inlineStr">
-        <is>
-          <t>3 / 1.8 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -2516,38 +2494,36 @@
       <c r="B8" s="2" t="inlineStr"/>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>1 / 1.4 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>6 / 2.1 / 1/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>2 / 1.3 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>1 / 0.3 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>7 / 4.7 / 2/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.1 / 0/8</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>0 / 0.0 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -2557,40 +2533,36 @@
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr"/>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>0 / 1.5 / 0/11</t>
-        </is>
+      <c r="C9" s="5" t="n">
+        <v>1</v>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>0 / 2.0 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>2 / 1.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>6 / 2.2 / 1/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>1 / 2.2 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>1 / 0.2 / 0/8</t>
-        </is>
-      </c>
-      <c r="I9" s="4" t="inlineStr">
-        <is>
-          <t>1 / 0.2 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -2600,40 +2572,36 @@
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr"/>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>0 / 1.5 / 0/11</t>
-        </is>
+      <c r="C10" s="3" t="n">
+        <v>2</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>1 / 0.5 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.2 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.3 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/8</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>0 / 0.0 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>55</v>
       </c>
     </row>
     <row r="11">
@@ -2642,44 +2610,40 @@
           <t>Cumbria - North</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>1 / 1.6 / 0/11</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>0 / 2.8 / 3/11</t>
-        </is>
+      <c r="B11" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>2</v>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.2 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/5</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -2689,40 +2653,38 @@
           <t>Cumbria - South</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>1 / 1.1 / 0/11</t>
-        </is>
+      <c r="B12" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="C12" s="2" t="inlineStr"/>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>1 / 0.7 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2 / 0.6 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.7 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>1 / 0.1 / 0/8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/5</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -2734,43 +2696,39 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>1 / 1.8 / 0/11</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>1 / 0.8 / 0/11</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>2</v>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.5 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/8</t>
-        </is>
-      </c>
-      <c r="I13" s="4" t="inlineStr">
-        <is>
-          <t>0 / 0.0 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -2780,40 +2738,36 @@
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr"/>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>0 / 0.4 / 0/11</t>
-        </is>
+      <c r="C14" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>3 / 2.5 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>2 / 0.6 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2 / 0.9 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>2 / 3.2 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/8</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>3 / 1.4 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -2823,35 +2777,33 @@
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr"/>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>0 / 0.1 / 0/11</t>
-        </is>
+      <c r="C15" s="5" t="n">
+        <v>1</v>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>5 / 3.2 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>3 / 2.1 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>6 / 1.2 / 1/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr"/>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>2 / 1.1 / 0/8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>3 / 1.0 / 0/5</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -2862,40 +2814,36 @@
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr"/>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>1 / 1.0 / 0/11</t>
-        </is>
+      <c r="C16" s="3" t="n">
+        <v>2</v>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>5 / 3.9 / 2/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.2 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>3 / 1.4 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>1 / 3.2 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/8</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>1 / 0.2 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="17">
@@ -2907,34 +2855,32 @@
       <c r="B17" s="4" t="inlineStr"/>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>1 / 0.7 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>5 / 2.1 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr"/>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>6 / 2.8 / 1/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>4 / 5.7 / 2/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>1 / 1.1 / 0/8</t>
-        </is>
-      </c>
-      <c r="I17" s="4" t="inlineStr">
-        <is>
-          <t>4 / 2.0 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="18">
@@ -2944,35 +2890,33 @@
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr"/>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>0 / 0.2 / 0/11</t>
-        </is>
+      <c r="C18" s="3" t="n">
+        <v>4</v>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>4 / 1.4 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>8 / 2.9 / 1/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr"/>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>2 / 1.2 / 0/8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>3 / 1.6 / 0/5</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -2983,28 +2927,24 @@
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr"/>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>2 / 1.3 / 0/11</t>
-        </is>
+      <c r="C19" s="5" t="n">
+        <v>2</v>
       </c>
       <c r="D19" s="4" t="inlineStr"/>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>3 / 3.9 / 2/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr"/>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>3 / 3.7 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr"/>
-      <c r="I19" s="4" t="inlineStr">
-        <is>
-          <t>3 / 2.2 / 0/5</t>
-        </is>
+      <c r="I19" s="5" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="20">
@@ -3013,45 +2953,41 @@
           <t>Greater Manchester - North</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>3 / 3.1 / 1/11</t>
-        </is>
+      <c r="B20" s="3" t="n">
+        <v>5</v>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.2 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.1 / 0/8</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>1 / 0.2 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="21">
@@ -3061,40 +2997,36 @@
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr"/>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>0 / 0.8 / 0/11</t>
-        </is>
+      <c r="C21" s="5" t="n">
+        <v>1</v>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>1 / 0.7 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>1 / 0.4 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>2 / 0.2 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/8</t>
-        </is>
-      </c>
-      <c r="I21" s="4" t="inlineStr">
-        <is>
-          <t>3 / 0.6 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="22">
@@ -3104,40 +3036,36 @@
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr"/>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>0 / 0.0 / 0/11</t>
-        </is>
+      <c r="C22" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>1 / 0.7 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>1 / 0.3 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.3 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>1 / 1.0 / 0/8</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>1 / 1.0 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="23">
@@ -3150,27 +3078,27 @@
       <c r="C23" s="4" t="inlineStr"/>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>14 / 7.4 / 7/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>0 / 1.7 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>10 / 5.0 / 2/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>1 / 2.8 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>4 / 3.5 / 0/8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr"/>
@@ -3181,44 +3109,42 @@
           <t>Herefordshire</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>0 / 1.4 / 0/11</t>
-        </is>
+      <c r="B24" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.2 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>1 / 0.1 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>0 / 1.2 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/5</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -3229,40 +3155,36 @@
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr"/>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>3 / 2.3 / 0/11</t>
-        </is>
+      <c r="C25" s="5" t="n">
+        <v>1</v>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>10 / 4.0 / 1/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>1 / 1.6 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>9 / 2.1 / 1/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>1 / 1.0 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>1 / 0.2 / 0/8</t>
-        </is>
-      </c>
-      <c r="I25" s="4" t="inlineStr">
-        <is>
-          <t>4 / 1.6 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="26">
@@ -3275,33 +3197,31 @@
       <c r="C26" s="2" t="inlineStr"/>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>8 / 4.5 / 1/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>3 / 4.3 / 2/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>7 / 2.8 / 1/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>1 / 3.2 / 1/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>2 / 1.6 / 0/8</t>
-        </is>
-      </c>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>2 / 0.8 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="27">
@@ -3310,44 +3230,42 @@
           <t>Lancashire - Blackpool &amp; Fylde</t>
         </is>
       </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>1 / 0.8 / 0/11</t>
-        </is>
+      <c r="B27" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>2 / 0.9 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>1 / 0.3 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/5</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -3357,45 +3275,39 @@
           <t>Lancashire - Central</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>3 / 2.8 / 0/11</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>0 / 0.2 / 0/11</t>
-        </is>
+      <c r="B28" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>1 / 0.3 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>1 / 0.5 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.2 / 0/8</t>
-        </is>
-      </c>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>0 / 0.0 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -3404,44 +3316,40 @@
           <t>Lancashire - East</t>
         </is>
       </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>3 / 2.5 / 0/11</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>0 / 0.7 / 0/11</t>
-        </is>
+      <c r="B29" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C29" s="5" t="n">
+        <v>3</v>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.3 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.2 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>3 / 1.1 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>1 / 1.2 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/5</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -3453,42 +3361,40 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>1 / 1.0 / 0/11</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>0 / 1.2 / 0/11</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="n">
+        <v>3</v>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/5</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -3500,42 +3406,42 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>0 / 1.3 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.1 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>1 / 1.2 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/5</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -3546,40 +3452,36 @@
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr"/>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>0 / 0.1 / 0/11</t>
-        </is>
+      <c r="C32" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>3 / 1.6 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>2 / 1.3 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>1 / 0.9 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>2 / 3.0 / 1/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>2 / 0.9 / 0/8</t>
-        </is>
-      </c>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t>3 / 3.0 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="33">
@@ -3589,40 +3491,36 @@
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr"/>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>0 / 1.7 / 0/11</t>
-        </is>
+      <c r="C33" s="5" t="n">
+        <v>2</v>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>4 / 1.2 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>3 / 1.6 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>3 / 2.7 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>1 / 2.8 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>1 / 1.4 / 0/8</t>
-        </is>
-      </c>
-      <c r="I33" s="4" t="inlineStr">
-        <is>
-          <t>2 / 1.0 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I33" s="5" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="34">
@@ -3638,7 +3536,7 @@
       <c r="F34" s="2" t="inlineStr"/>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>10 / 5.2 / 2/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr"/>
@@ -3651,40 +3549,36 @@
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr"/>
-      <c r="C35" s="4" t="inlineStr">
-        <is>
-          <t>0 / 0.4 / 0/11</t>
-        </is>
+      <c r="C35" s="5" t="n">
+        <v>2</v>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.3 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>1 / 0.4 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>6 / 2.0 / 1/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>1 / 0.5 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.1 / 0/8</t>
-        </is>
-      </c>
-      <c r="I35" s="4" t="inlineStr">
-        <is>
-          <t>0 / 0.0 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I35" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -3695,42 +3589,40 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.1 / 0/10</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>0 / 0.0 / 0/10</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/5</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -3742,42 +3634,42 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>1 / 2.0 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>1 / 0.8 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>1 / 1.7 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/5</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -3787,45 +3679,39 @@
           <t>Merseyside - Wirral</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>1 / 1.5 / 0/11</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>0 / 0.5 / 0/11</t>
-        </is>
+      <c r="B38" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C38" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>1 / 1.0 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>1 / 0.3 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>3 / 0.6 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>1 / 0.2 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/8</t>
-        </is>
-      </c>
-      <c r="I38" s="2" t="inlineStr">
-        <is>
-          <t>1 / 1.0 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="39">
@@ -3835,36 +3721,32 @@
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr"/>
-      <c r="C39" s="4" t="inlineStr">
-        <is>
-          <t>0 / 1.1 / 0/11</t>
-        </is>
+      <c r="C39" s="5" t="n">
+        <v>2</v>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.7 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr"/>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>2 / 1.6 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>2 / 4.2 / 2/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.2 / 0/8</t>
-        </is>
-      </c>
-      <c r="I39" s="4" t="inlineStr">
-        <is>
-          <t>1 / 0.8 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I39" s="5" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="40">
@@ -3878,24 +3760,22 @@
       <c r="D40" s="2" t="inlineStr"/>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.9 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>6 / 4.1 / 1/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr"/>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>1 / 1.1 / 0/8</t>
-        </is>
-      </c>
-      <c r="I40" s="2" t="inlineStr">
-        <is>
-          <t>4 / 2.4 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="n">
+        <v>75</v>
       </c>
     </row>
     <row r="41">
@@ -3904,44 +3784,40 @@
           <t>North Scotland</t>
         </is>
       </c>
-      <c r="B41" s="4" t="inlineStr">
-        <is>
-          <t>6 / 5.6 / 4/10</t>
-        </is>
-      </c>
-      <c r="C41" s="4" t="inlineStr">
-        <is>
-          <t>0 / 0.0 / 0/10</t>
-        </is>
+      <c r="B41" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>6 / 3.0 / 1/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.2 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>1 / 1.5 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/5</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -3951,45 +3827,39 @@
           <t>North Wales - East</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>5 / 4.5 / 1/10</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>0 / 0.2 / 0/10</t>
-        </is>
+      <c r="B42" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C42" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>1 / 1.3 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>1 / 0.4 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>1 / 1.5 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/8</t>
-        </is>
-      </c>
-      <c r="I42" s="2" t="inlineStr">
-        <is>
-          <t>1 / 1.0 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I42" s="3" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="43">
@@ -4000,43 +3870,39 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>3 / 1.8 / 0/10</t>
-        </is>
-      </c>
-      <c r="C43" s="4" t="inlineStr">
-        <is>
-          <t>0 / 0.0 / 0/10</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>1 / 0.2 / 0/8</t>
-        </is>
-      </c>
-      <c r="I43" s="4" t="inlineStr">
-        <is>
-          <t>1 / 0.4 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I43" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -4046,40 +3912,36 @@
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr"/>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>0 / 0.0 / 0/11</t>
-        </is>
+      <c r="C44" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>11 / 3.6 / 1/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>1 / 1.3 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>6 / 2.2 / 1/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>2 / 3.3 / 2/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>3 / 2.5 / 1/8</t>
-        </is>
-      </c>
-      <c r="I44" s="2" t="inlineStr">
-        <is>
-          <t>1 / 0.2 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I44" s="3" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="45">
@@ -4089,35 +3951,33 @@
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr"/>
-      <c r="C45" s="4" t="inlineStr">
-        <is>
-          <t>1 / 1.8 / 0/10</t>
-        </is>
+      <c r="C45" s="5" t="n">
+        <v>1</v>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>1 / 1.2 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr"/>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.1 / 0/8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>1 / 1.0 / 0/5</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -4127,45 +3987,41 @@
           <t>Northern Ireland - West</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>4 / 4.1 / 0/10</t>
-        </is>
+      <c r="B46" s="3" t="n">
+        <v>2</v>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>3 / 1.0 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.2 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/8</t>
-        </is>
-      </c>
-      <c r="I46" s="2" t="inlineStr">
-        <is>
-          <t>0 / 0.0 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I46" s="3" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="47">
@@ -4175,36 +4031,32 @@
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr"/>
-      <c r="C47" s="4" t="inlineStr">
-        <is>
-          <t>1 / 0.5 / 0/11</t>
-        </is>
+      <c r="C47" s="5" t="n">
+        <v>1</v>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>3 / 1.8 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>2 / 2.1 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>4 / 2.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t>1 / 3.7 / 2/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H47" s="4" t="inlineStr"/>
-      <c r="I47" s="4" t="inlineStr">
-        <is>
-          <t>1 / 1.0 / 0/5</t>
-        </is>
+      <c r="I47" s="5" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="48">
@@ -4217,33 +4069,31 @@
       <c r="C48" s="2" t="inlineStr"/>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>5 / 3.0 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>2 / 1.7 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>10 / 4.6 / 2/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>1 / 2.8 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>1 / 0.2 / 0/8</t>
-        </is>
-      </c>
-      <c r="I48" s="2" t="inlineStr">
-        <is>
-          <t>3 / 0.8 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I48" s="3" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="49">
@@ -4254,42 +4104,42 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H49" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I49" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/5</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -4301,42 +4151,42 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>2 / 1.1 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>1 / 0.2 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/5</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -4347,40 +4197,36 @@
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr"/>
-      <c r="C51" s="4" t="inlineStr">
-        <is>
-          <t>0 / 0.1 / 0/10</t>
-        </is>
+      <c r="C51" s="5" t="n">
+        <v>1</v>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>4 / 2.2 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>4 / 2.4 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>1 / 0.1 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr">
         <is>
-          <t>1 / 1.2 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H51" s="4" t="inlineStr">
         <is>
-          <t>1 / 0.4 / 0/8</t>
-        </is>
-      </c>
-      <c r="I51" s="4" t="inlineStr">
-        <is>
-          <t>1 / 0.2 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I51" s="5" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="52">
@@ -4389,45 +4235,39 @@
           <t>Scotland Central - Falkirk &amp; Stirling</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>2 / 2.8 / 0/10</t>
-        </is>
-      </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>0 / 0.0 / 0/10</t>
-        </is>
+      <c r="B52" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>1 / 1.2 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/8</t>
-        </is>
-      </c>
-      <c r="I52" s="2" t="inlineStr">
-        <is>
-          <t>0 / 0.0 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I52" s="3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="53">
@@ -4438,42 +4278,40 @@
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>2 / 1.5 / 0/10</t>
-        </is>
-      </c>
-      <c r="C53" s="4" t="inlineStr">
-        <is>
-          <t>0 / 0.0 / 0/10</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>2 / 1.0 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.7 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H53" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I53" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/5</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -4483,44 +4321,42 @@
           <t>Scotland Central - Tayside</t>
         </is>
       </c>
-      <c r="B54" s="2" t="inlineStr">
-        <is>
-          <t>5 / 3.8 / 0/10</t>
-        </is>
+      <c r="B54" s="3" t="n">
+        <v>4</v>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.2 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>1 / 1.2 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.2 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.7 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>1 / 0.2 / 0/5</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -4532,43 +4368,41 @@
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>1 / 0.5 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>1 / 0.4 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G55" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H55" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/8</t>
-        </is>
-      </c>
-      <c r="I55" s="4" t="inlineStr">
-        <is>
-          <t>1 / 0.6 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I55" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="56">
@@ -4578,40 +4412,36 @@
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr"/>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>0 / 0.0 / 0/10</t>
-        </is>
+      <c r="C56" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>4 / 3.1 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.2 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.2 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.3 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.6 / 0/8</t>
-        </is>
-      </c>
-      <c r="I56" s="2" t="inlineStr">
-        <is>
-          <t>3 / 2.4 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I56" s="3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="57">
@@ -4620,45 +4450,41 @@
           <t>Scotland West - Lanarkshire</t>
         </is>
       </c>
-      <c r="B57" s="4" t="inlineStr">
-        <is>
-          <t>0 / 0.5 / 0/10</t>
-        </is>
+      <c r="B57" s="5" t="n">
+        <v>1</v>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.1 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.4 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F57" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H57" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/8</t>
-        </is>
-      </c>
-      <c r="I57" s="4" t="inlineStr">
-        <is>
-          <t>0 / 0.0 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I57" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="58">
@@ -4669,43 +4495,39 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>1 / 1.0 / 0/10</t>
-        </is>
-      </c>
-      <c r="C58" s="2" t="inlineStr">
-        <is>
-          <t>0 / 0.0 / 0/10</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>1 / 0.4 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.7 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/8</t>
-        </is>
-      </c>
-      <c r="I58" s="2" t="inlineStr">
-        <is>
-          <t>0 / 0.0 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I58" s="3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="59">
@@ -4715,35 +4537,33 @@
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr"/>
-      <c r="C59" s="4" t="inlineStr">
-        <is>
-          <t>0 / 1.8 / 0/11</t>
-        </is>
+      <c r="C59" s="5" t="n">
+        <v>3</v>
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>0 / 1.1 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>2 / 1.7 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t>1 / 0.3 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G59" s="4" t="inlineStr"/>
       <c r="H59" s="4" t="inlineStr">
         <is>
-          <t>2 / 1.9 / 0/8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I59" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/5</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -4754,40 +4574,36 @@
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr"/>
-      <c r="C60" s="2" t="inlineStr">
-        <is>
-          <t>1 / 3.5 / 3/11</t>
-        </is>
+      <c r="C60" s="3" t="n">
+        <v>4</v>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>2 / 1.3 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>1 / 0.3 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>4 / 0.6 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>2 / 3.3 / 1/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.1 / 0/8</t>
-        </is>
-      </c>
-      <c r="I60" s="2" t="inlineStr">
-        <is>
-          <t>2 / 0.4 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I60" s="3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="61">
@@ -4797,34 +4613,32 @@
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr"/>
-      <c r="C61" s="4" t="inlineStr">
-        <is>
-          <t>0 / 0.2 / 0/11</t>
-        </is>
+      <c r="C61" s="5" t="n">
+        <v>3</v>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>1 / 1.4 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t>2 / 1.2 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
-          <t>3 / 2.5 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H61" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.1 / 0/8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I61" s="4" t="inlineStr"/>
@@ -4836,35 +4650,33 @@
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr"/>
-      <c r="C62" s="2" t="inlineStr">
-        <is>
-          <t>0 / 0.9 / 0/11</t>
-        </is>
+      <c r="C62" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>3 / 1.6 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr"/>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2 / 0.3 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>1 / 1.8 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>1 / 1.0 / 0/8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>1 / 0.4 / 0/5</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -4878,23 +4690,23 @@
       <c r="C63" s="4" t="inlineStr"/>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>6 / 4.5 / 4/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>5 / 4.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F63" s="4" t="inlineStr"/>
       <c r="G63" s="4" t="inlineStr">
         <is>
-          <t>5 / 5.2 / 2/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H63" s="4" t="inlineStr">
         <is>
-          <t>3 / 2.0 / 0/8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I63" s="4" t="inlineStr"/>
@@ -4909,33 +4721,31 @@
       <c r="C64" s="2" t="inlineStr"/>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>7 / 3.6 / 1/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>4 / 2.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>5 / 2.6 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>4 / 4.2 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>6 / 5.8 / 6/8</t>
-        </is>
-      </c>
-      <c r="I64" s="2" t="inlineStr">
-        <is>
-          <t>4 / 2.8 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I64" s="3" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="65">
@@ -4946,43 +4756,41 @@
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.1 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F65" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G65" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H65" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/8</t>
-        </is>
-      </c>
-      <c r="I65" s="4" t="inlineStr">
-        <is>
-          <t>0 / 0.0 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I65" s="5" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="66">
@@ -4991,44 +4799,40 @@
           <t>Wales - West</t>
         </is>
       </c>
-      <c r="B66" s="2" t="inlineStr">
-        <is>
-          <t>3 / 1.9 / 0/10</t>
-        </is>
-      </c>
-      <c r="C66" s="2" t="inlineStr">
-        <is>
-          <t>0 / 0.0 / 0/10</t>
-        </is>
+      <c r="B66" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C66" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.7 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.1 / 0/8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/5</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -5038,44 +4842,40 @@
           <t>Wales South - Cardiff &amp; Vale</t>
         </is>
       </c>
-      <c r="B67" s="4" t="inlineStr">
-        <is>
-          <t>5 / 4.1 / 1/10</t>
-        </is>
-      </c>
-      <c r="C67" s="4" t="inlineStr">
-        <is>
-          <t>0 / 0.0 / 0/10</t>
-        </is>
+      <c r="B67" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C67" s="5" t="n">
+        <v>1</v>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>3 / 1.7 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>2 / 1.3 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F67" s="4" t="inlineStr">
         <is>
-          <t>2 / 0.9 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G67" s="4" t="inlineStr">
         <is>
-          <t>0 / 1.2 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H67" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I67" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/5</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -5087,42 +4887,42 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>1 / 2.7 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.1 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>1 / 0.3 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>2 / 1.3 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.7 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/5</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -5132,45 +4932,39 @@
           <t>Wales South - Swansea Bay</t>
         </is>
       </c>
-      <c r="B69" s="4" t="inlineStr">
-        <is>
-          <t>1 / 2.9 / 1/10</t>
-        </is>
-      </c>
-      <c r="C69" s="4" t="inlineStr">
-        <is>
-          <t>0 / 0.1 / 0/10</t>
-        </is>
+      <c r="B69" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C69" s="5" t="n">
+        <v>1</v>
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>1 / 1.8 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>1 / 0.7 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F69" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G69" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.3 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H69" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/8</t>
-        </is>
-      </c>
-      <c r="I69" s="4" t="inlineStr">
-        <is>
-          <t>0 / 0.0 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I69" s="5" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="70">
@@ -5181,43 +4975,39 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>2 / 1.4 / 1/10</t>
-        </is>
-      </c>
-      <c r="C70" s="2" t="inlineStr">
-        <is>
-          <t>0 / 0.0 / 0/10</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.3 / 0/10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>4 / 2.6 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.4 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.2 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/8</t>
-        </is>
-      </c>
-      <c r="I70" s="2" t="inlineStr">
-        <is>
-          <t>0 / 0.0 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I70" s="3" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="71">
@@ -5229,30 +5019,28 @@
       <c r="B71" s="4" t="inlineStr"/>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>1 / 1.0 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>11 / 4.0 / 1/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>3 / 3.9 / 2/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F71" s="4" t="inlineStr"/>
       <c r="G71" s="4" t="inlineStr">
         <is>
-          <t>3 / 2.7 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H71" s="4" t="inlineStr"/>
-      <c r="I71" s="4" t="inlineStr">
-        <is>
-          <t>5 / 3.4 / 0/5</t>
-        </is>
+      <c r="I71" s="5" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="72">
@@ -5262,39 +5050,37 @@
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr"/>
-      <c r="C72" s="2" t="inlineStr">
-        <is>
-          <t>1 / 1.1 / 0/11</t>
-        </is>
+      <c r="C72" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>1 / 1.0 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>3 / 1.1 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>1 / 0.4 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>1 / 1.3 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>1 / 1.0 / 0/5</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -5305,40 +5091,36 @@
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr"/>
-      <c r="C73" s="4" t="inlineStr">
-        <is>
-          <t>0 / 0.0 / 0/11</t>
-        </is>
+      <c r="C73" s="5" t="n">
+        <v>4</v>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>6 / 1.3 / 1/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>1 / 0.6 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F73" s="4" t="inlineStr">
         <is>
-          <t>5 / 2.4 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G73" s="4" t="inlineStr">
         <is>
-          <t>3 / 2.2 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H73" s="4" t="inlineStr">
         <is>
-          <t>3 / 3.1 / 0/8</t>
-        </is>
-      </c>
-      <c r="I73" s="4" t="inlineStr">
-        <is>
-          <t>2 / 0.4 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I73" s="5" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="74">
@@ -5351,33 +5133,31 @@
       <c r="C74" s="2" t="inlineStr"/>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>3 / 2.0 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>4 / 3.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>3 / 1.1 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>0 / 2.7 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.6 / 0/8</t>
-        </is>
-      </c>
-      <c r="I74" s="2" t="inlineStr">
-        <is>
-          <t>1 / 1.0 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I74" s="3" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="75">
@@ -5387,40 +5167,36 @@
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr"/>
-      <c r="C75" s="4" t="inlineStr">
-        <is>
-          <t>0 / 1.3 / 0/11</t>
-        </is>
+      <c r="C75" s="5" t="n">
+        <v>2</v>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>1 / 2.1 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>2 / 0.4 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F75" s="4" t="inlineStr">
         <is>
-          <t>3 / 1.6 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G75" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.8 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H75" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.2 / 0/8</t>
-        </is>
-      </c>
-      <c r="I75" s="4" t="inlineStr">
-        <is>
-          <t>1 / 0.4 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I75" s="5" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="76">
@@ -5430,40 +5206,36 @@
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr"/>
-      <c r="C76" s="2" t="inlineStr">
-        <is>
-          <t>0 / 0.7 / 0/11</t>
-        </is>
+      <c r="C76" s="3" t="n">
+        <v>3</v>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>0 / 1.2 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>2 / 1.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2 / 0.4 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>2 / 4.0 / 0/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>1 / 1.2 / 0/8</t>
-        </is>
-      </c>
-      <c r="I76" s="2" t="inlineStr">
-        <is>
-          <t>4 / 2.8 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I76" s="3" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="77">
@@ -5473,36 +5245,32 @@
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr"/>
-      <c r="C77" s="4" t="inlineStr">
-        <is>
-          <t>1 / 3.5 / 0/11</t>
-        </is>
+      <c r="C77" s="5" t="n">
+        <v>4</v>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>3 / 0.9 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>0 / 0.1 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F77" s="4" t="inlineStr">
         <is>
-          <t>12 / 2.7 / 1/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G77" s="4" t="inlineStr"/>
       <c r="H77" s="4" t="inlineStr">
         <is>
-          <t>2 / 1.5 / 0/8</t>
-        </is>
-      </c>
-      <c r="I77" s="4" t="inlineStr">
-        <is>
-          <t>2 / 1.0 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I77" s="5" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="78">
@@ -5515,33 +5283,31 @@
       <c r="C78" s="2" t="inlineStr"/>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>4 / 2.0 / 0/11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>4 / 3.1 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>6 / 2.0 / 1/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>0 / 2.3 / 2/6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/8</t>
-        </is>
-      </c>
-      <c r="I78" s="2" t="inlineStr">
-        <is>
-          <t>2 / 1.0 / 0/5</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I78" s="3" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="79">
@@ -5555,20 +5321,18 @@
       <c r="D79" s="4" t="inlineStr"/>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>4 / 4.0 / 0/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F79" s="4" t="inlineStr">
         <is>
-          <t>15 / 5.4 / 3/9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G79" s="4" t="inlineStr"/>
       <c r="H79" s="4" t="inlineStr"/>
-      <c r="I79" s="4" t="inlineStr">
-        <is>
-          <t>3 / 2.6 / 0/5</t>
-        </is>
+      <c r="I79" s="5" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>